<commit_message>
Use exact per-order column widths for 25.08
Pulled the real widths from the kitchen's own 25.08 tab: exception
columns are 14.63 but the two "ОСНОВНОЙ ЗАКАЗ" columns are wider
(15.5 premium, 16.13 standard) - not uniform like 22.08's reference.
build_xlsx.py now checks an optional order.COL_WIDTHS override before
falling back to the sheet-wide default.
</commit_message>
<xml_diff>
--- a/output/Гонконг 25.08.2026 (обработка).xlsx
+++ b/output/Гонконг 25.08.2026 (обработка).xlsx
@@ -522,14 +522,14 @@
     <col width="17.63" customWidth="1" min="5" max="5"/>
     <col width="14.63" customWidth="1" min="6" max="6"/>
     <col width="14.63" customWidth="1" min="7" max="7"/>
-    <col width="12.6328125" customWidth="1" min="8" max="8"/>
-    <col width="12.6328125" customWidth="1" min="9" max="9"/>
-    <col width="12.6328125" customWidth="1" min="10" max="10"/>
-    <col width="12.6328125" customWidth="1" min="11" max="11"/>
-    <col width="12.6328125" customWidth="1" min="12" max="12"/>
-    <col width="12.6328125" customWidth="1" min="13" max="13"/>
-    <col width="12.6328125" customWidth="1" min="14" max="14"/>
-    <col width="12.6328125" customWidth="1" min="15" max="15"/>
+    <col width="14.63" customWidth="1" min="8" max="8"/>
+    <col width="14.63" customWidth="1" min="9" max="9"/>
+    <col width="15.5" customWidth="1" min="10" max="10"/>
+    <col width="16.13" customWidth="1" min="11" max="11"/>
+    <col width="14.63" customWidth="1" min="12" max="12"/>
+    <col width="14.63" customWidth="1" min="13" max="13"/>
+    <col width="14.63" customWidth="1" min="14" max="14"/>
+    <col width="14.63" customWidth="1" min="15" max="15"/>
   </cols>
   <sheetData>
     <row r="1" ht="32.25" customHeight="1">

</xml_diff>